<commit_message>
Atualiza lista de pintura do Display Aramado G
</commit_message>
<xml_diff>
--- a/PINTURA/LISTA PINTURA DISPLAY ARAMADO G.xlsx
+++ b/PINTURA/LISTA PINTURA DISPLAY ARAMADO G.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS---BACKEND-IA\PINTURA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD04262C-C999-48CE-95B6-A1A3095CB452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58938A93-2276-42CB-8297-2F41C43AD1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4635" yWindow="5505" windowWidth="38700" windowHeight="14475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="29">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -65,34 +65,64 @@
     <t>PINTURA</t>
   </si>
   <si>
-    <t>ENVIO - VERMELHO</t>
-  </si>
-  <si>
-    <t>ENVIO - AMARELO</t>
-  </si>
-  <si>
-    <t>ENVIO - MARROM</t>
-  </si>
-  <si>
-    <t>ENVIO - PRETO</t>
-  </si>
-  <si>
-    <t>ENVIO - BORDO</t>
-  </si>
-  <si>
-    <t>RETORNO - VERMELHO</t>
-  </si>
-  <si>
-    <t>RETORNO - AMARELO</t>
-  </si>
-  <si>
-    <t>RETORNO - MARROM</t>
-  </si>
-  <si>
-    <t>RETORNO - PRETO</t>
-  </si>
-  <si>
-    <t>RETORNO - BORDO</t>
+    <t>CORPO ENVIO - VERMELHO</t>
+  </si>
+  <si>
+    <t>CORPO ENVIO - AMARELO</t>
+  </si>
+  <si>
+    <t>CORPO ENVIO - MARROM</t>
+  </si>
+  <si>
+    <t>CORPO ENVIO - PRETO</t>
+  </si>
+  <si>
+    <t>CORPO ENVIO - BORDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CORPO RETORNO - VERMELHO</t>
+  </si>
+  <si>
+    <t>CORPO RETORNO - AMARELO</t>
+  </si>
+  <si>
+    <t>CORPO RETORNO - MARROM</t>
+  </si>
+  <si>
+    <t>CORPO RETORNO - PRETO</t>
+  </si>
+  <si>
+    <t>CORPO RETORNO - BORDO</t>
+  </si>
+  <si>
+    <t>TESTEIRA ENVIO - VERMELHO</t>
+  </si>
+  <si>
+    <t>TESTEIRA ENVIO - AMARELO</t>
+  </si>
+  <si>
+    <t>TESTEIRA ENVIO - MARROM</t>
+  </si>
+  <si>
+    <t>TESTEIRA ENVIO - PRETO</t>
+  </si>
+  <si>
+    <t>TESTEIRA ENVIO - BORDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TESTEIRA RETORNO - VERMELHO</t>
+  </si>
+  <si>
+    <t>TESTEIRA RETORNO - AMARELO</t>
+  </si>
+  <si>
+    <t>TESTEIRA RETORNO - MARROM</t>
+  </si>
+  <si>
+    <t>TESTEIRA RETORNO - PRETO</t>
+  </si>
+  <si>
+    <t>TESTEIRA RETORNO - BORDO</t>
   </si>
 </sst>
 </file>
@@ -648,51 +678,223 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E12" s="1"/>
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>476</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E13" s="1"/>
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <f>201+60</f>
+        <v>261</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E14" s="1"/>
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>85</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E15" s="1"/>
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>322</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <f>201+60</f>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E27" s="1"/>
     </row>
   </sheetData>

</xml_diff>